<commit_message>
Resolving git issues and failing ui tests
</commit_message>
<xml_diff>
--- a/src/test/resources/data/loginTestDataPW.xlsx
+++ b/src/test/resources/data/loginTestDataPW.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20417"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D627DBC3-9E1A-4A2F-9543-C7DB614EBA14}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3055697D-2C74-4CC6-8DAD-4FAE9B02807A}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -65,10 +65,10 @@
     <t>te</t>
   </si>
   <si>
-    <t>natashatestpw@gmail.com</t>
-  </si>
-  <si>
-    <t>3230474N5a5t5e5!</t>
+    <t>customer@practicesoftwaretesting.com</t>
+  </si>
+  <si>
+    <t>welcome01</t>
   </si>
 </sst>
 </file>

</xml_diff>